<commit_message>
Actualizacion records 29/06/2026 12:07:10,79
</commit_message>
<xml_diff>
--- a/data/50m_Femenino_Absoluto_Braza.xlsx
+++ b/data/50m_Femenino_Absoluto_Braza.xlsx
@@ -464,13 +464,13 @@
         <v>C.N. MEDITERRANEO VALENCIA</v>
       </c>
       <c r="F2" t="str">
-        <v>00:00:36.07</v>
+        <v>00:00:36.06</v>
       </c>
       <c r="G2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="H2" s="1">
-        <v>46081.99949074074</v>
+        <v>46200.99949074074</v>
       </c>
       <c r="I2" t="str">
         <v>Deportista</v>
@@ -482,10 +482,10 @@
         <v>Electrónico</v>
       </c>
       <c r="L2" t="str">
-        <v>CAMPEONATO AUTONOMICO INFANTIL DE INVIERNO 2026</v>
+        <v>CAMPEONATO AUTONOMICO INFANTIL DE VERANO DE LA C.V. 2026</v>
       </c>
       <c r="M2" t="str">
-        <v>CASTELLÓN</v>
+        <v>CASTELLON</v>
       </c>
       <c r="N2" t="str">
         <v>No</v>

</xml_diff>